<commit_message>
Update data files: VC, VC credit conso, EDC, Code Magasin + add CREDIT PARTICULIER
</commit_message>
<xml_diff>
--- a/2025/Code MAGASIN Business Central.xlsx
+++ b/2025/Code MAGASIN Business Central.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mgonline-my.sharepoint.com/personal/hamadi_chkondali_smg_com_tn/Documents/Documents/hamadi/grands compte/hamadi/dashbord convention/table vente/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{D558B66C-BBCD-4D84-A823-F8D869F06087}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C252BEBC-4D7D-4CF1-8E85-276EFE084ABC}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="8_{D558B66C-BBCD-4D84-A823-F8D869F06087}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0836EBA-AE3C-4746-A782-5009476270AA}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="2420" yWindow="2420" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>

</xml_diff>